<commit_message>
add global filter in macro sheet (but not yet implemented)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping.xlsx
+++ b/tests/testthat/excel/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\questabber\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42CA5DAF-BEEB-4ACC-A0B8-233C79ED5D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38121C9A-BCD7-4532-B641-4BC23F985631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="273">
   <si>
     <t>Make script</t>
   </si>
@@ -877,6 +877,9 @@
   <si>
     <t>1 2</t>
   </si>
+  <si>
+    <t>id != 100</t>
+  </si>
 </sst>
 </file>
 
@@ -3082,7 +3085,9 @@
       <c r="D9" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="E9" s="14"/>
+      <c r="E9" s="14" t="s">
+        <v>272</v>
+      </c>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>

</xml_diff>

<commit_message>
rename: - RowVars to RowVar - ColVars to ColVar (as before)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping.xlsx
+++ b/tests/testthat/excel/mapping.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\questabber\tests\testthat\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38121C9A-BCD7-4532-B641-4BC23F985631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D19B08-12F6-4408-80E7-9A2F0F26265B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
     <definedName name="V_ScenName">Config!$C$16</definedName>
     <definedName name="V_TemplatePath">Config!$B$26</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -512,9 +512,6 @@
     <t>Scenario 50</t>
   </si>
   <si>
-    <t>ColVars</t>
-  </si>
-  <si>
     <t>Header variables</t>
   </si>
   <si>
@@ -755,9 +752,6 @@
     <t>Type</t>
   </si>
   <si>
-    <t>RowVars</t>
-  </si>
-  <si>
     <t>Filter</t>
   </si>
   <si>
@@ -880,6 +874,12 @@
   <si>
     <t>id != 100</t>
   </si>
+  <si>
+    <t>RowVar</t>
+  </si>
+  <si>
+    <t>ColVar</t>
+  </si>
 </sst>
 </file>
 
@@ -939,7 +939,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1018,6 +1018,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1032,7 +1038,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1076,6 +1082,7 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2516,19 +2523,19 @@
     </row>
     <row r="5" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A5" s="28" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B5" s="20" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="D5" s="20" t="s">
         <v>152</v>
       </c>
-      <c r="D5" s="20" t="s">
-        <v>153</v>
-      </c>
       <c r="E5" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
@@ -2583,16 +2590,16 @@
     </row>
     <row r="6" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A6" s="28" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B6" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="D6" s="20" t="s">
         <v>156</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>157</v>
       </c>
       <c r="E6" s="14">
         <v>-1</v>
@@ -2748,13 +2755,13 @@
     </row>
     <row r="7" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="C7" s="20" t="s">
         <v>159</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>160</v>
       </c>
       <c r="D7" s="20"/>
       <c r="E7" s="14">
@@ -2911,13 +2918,13 @@
     </row>
     <row r="8" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="B8" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>162</v>
-      </c>
       <c r="C8" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D8" s="20"/>
       <c r="E8" s="14">
@@ -3074,19 +3081,19 @@
     </row>
     <row r="9" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B9" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="D9" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="D9" s="20" t="s">
-        <v>165</v>
-      </c>
       <c r="E9" s="14" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
@@ -3198,14 +3205,14 @@
     </row>
     <row r="11" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="B11" s="20" t="s">
         <v>166</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>167</v>
       </c>
       <c r="C11" s="20"/>
       <c r="D11" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
@@ -3261,11 +3268,11 @@
     </row>
     <row r="12" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D12" s="20"/>
       <c r="E12" s="14"/>
@@ -3322,10 +3329,10 @@
     </row>
     <row r="13" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>170</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>171</v>
       </c>
       <c r="C13" s="20"/>
       <c r="D13" s="20"/>
@@ -3383,11 +3390,11 @@
     </row>
     <row r="14" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D14" s="20"/>
       <c r="E14" s="14"/>
@@ -3444,10 +3451,10 @@
     </row>
     <row r="15" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>173</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>174</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
@@ -3505,14 +3512,14 @@
     </row>
     <row r="16" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B16" s="20"/>
       <c r="C16" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E16" s="14"/>
       <c r="F16" s="14"/>
@@ -3568,10 +3575,10 @@
     </row>
     <row r="17" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="B17" s="20" t="s">
         <v>177</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>178</v>
       </c>
       <c r="C17" s="20"/>
       <c r="D17" s="20"/>
@@ -3629,335 +3636,335 @@
     </row>
     <row r="18" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="B18" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="C18" s="20" t="s">
         <v>180</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>181</v>
       </c>
       <c r="D18" s="20"/>
       <c r="E18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="L18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="O18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="P18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Q18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="R18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="S18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="T18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="U18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="V18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="W18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="X18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Y18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="Z18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AA18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AB18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AC18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AD18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AE18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AF18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AG18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AH18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AI18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AJ18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AK18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AL18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AM18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AN18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AO18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AP18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AQ18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AR18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AS18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AT18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AU18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AV18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AW18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AX18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AY18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AZ18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="BA18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="BB18" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="BD18" s="19"/>
     </row>
     <row r="19" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D19" s="20"/>
       <c r="E19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="L19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="M19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="N19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="O19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="P19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Q19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="R19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="S19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="T19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="U19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="V19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="W19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="X19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Y19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Z19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AA19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AB19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AC19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AD19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AE19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AF19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AG19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AH19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AI19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AJ19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AK19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AL19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AM19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AN19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AO19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AP19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AQ19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AR19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AS19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AT19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AU19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AV19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AW19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AX19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AY19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AZ19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="BA19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="BB19" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="BD19" s="19"/>
     </row>
     <row r="20" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D20" s="20"/>
       <c r="E20" s="14"/>
@@ -4014,175 +4021,175 @@
     </row>
     <row r="21" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="B21" s="20" t="s">
         <v>186</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>187</v>
       </c>
       <c r="C21" s="20"/>
       <c r="D21" s="20"/>
       <c r="E21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="O21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="Q21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="R21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="S21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="T21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="U21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="V21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="W21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="X21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="Y21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="Z21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AA21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AB21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AC21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AD21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AE21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AF21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AG21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AH21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AI21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AJ21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AK21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AL21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AM21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AN21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AO21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AP21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AQ21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AR21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AS21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AT21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AU21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AV21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AW21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AX21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AY21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AZ21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="BA21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="BB21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="BD21" s="19"/>
     </row>
     <row r="22" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="B22" s="20" t="s">
         <v>189</v>
-      </c>
-      <c r="B22" s="20" t="s">
-        <v>190</v>
       </c>
       <c r="C22" s="20"/>
       <c r="D22" s="20" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E22" s="14"/>
       <c r="F22" s="14"/>
@@ -4238,11 +4245,11 @@
     </row>
     <row r="23" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B23" s="20"/>
       <c r="C23" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D23" s="20"/>
       <c r="E23" s="14"/>
@@ -4299,11 +4306,11 @@
     </row>
     <row r="24" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B24" s="20"/>
       <c r="C24" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D24" s="20"/>
       <c r="E24" s="14"/>
@@ -4360,11 +4367,11 @@
     </row>
     <row r="25" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B25" s="20"/>
       <c r="C25" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D25" s="20"/>
       <c r="E25" s="14"/>
@@ -4421,11 +4428,11 @@
     </row>
     <row r="26" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B26" s="20"/>
       <c r="C26" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D26" s="20"/>
       <c r="E26" s="14"/>
@@ -4482,498 +4489,498 @@
     </row>
     <row r="27" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D27" s="20"/>
       <c r="E27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="N27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="P27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Q27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="R27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="S27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="T27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="U27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="V27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="W27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="X27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Y27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Z27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AA27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AB27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AC27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AD27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AE27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AF27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AG27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AH27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AI27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AJ27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AK27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AL27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AM27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AN27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AO27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AP27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AQ27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AR27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AS27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AT27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AU27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AV27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AW27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AX27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AY27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AZ27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="BA27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="BB27" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="BD27" s="19"/>
     </row>
     <row r="28" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="B28" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="C28" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="D28" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="E28" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="E28" s="14" t="s">
-        <v>202</v>
-      </c>
       <c r="F28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="L28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="M28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="N28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="O28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="P28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Q28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="R28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="S28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="T28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="U28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="V28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="W28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="X28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Y28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Z28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AA28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AB28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AC28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AD28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AE28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AF28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AG28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AH28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AI28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AJ28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AK28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AL28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AM28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AN28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AO28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AP28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AQ28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AR28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AS28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AT28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AU28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AV28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AW28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AX28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AY28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AZ28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="BA28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="BB28" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="BD28" s="19"/>
     </row>
     <row r="29" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B29" s="20"/>
       <c r="C29" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D29" s="20"/>
       <c r="E29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="M29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="N29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="O29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="P29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="Q29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="R29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="S29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="T29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="U29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="V29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="W29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="X29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="Y29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="Z29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AA29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AB29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AC29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AD29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AE29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AF29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AG29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AH29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AI29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AJ29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AK29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AL29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AM29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AN29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AO29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AP29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AQ29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AR29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AS29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AT29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AU29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AV29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AW29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AX29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AY29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AZ29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="BA29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="BB29" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="BD29" s="19"/>
     </row>
     <row r="30" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D30" s="20"/>
       <c r="E30" s="14"/>
@@ -5030,176 +5037,176 @@
     </row>
     <row r="31" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="B31" s="20" t="s">
         <v>206</v>
       </c>
-      <c r="B31" s="20" t="s">
-        <v>207</v>
-      </c>
       <c r="C31" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D31" s="20"/>
       <c r="E31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="L31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="M31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="N31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="O31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="P31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="R31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="S31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="T31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="U31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="V31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="W31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="X31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Y31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Z31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AA31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AB31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AC31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AD31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AE31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AF31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AG31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AH31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AI31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AJ31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AK31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AL31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AM31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AN31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AO31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AP31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AQ31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AR31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AS31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AT31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AU31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AV31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AW31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AX31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AY31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AZ31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="BA31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="BB31" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="BD31" s="19"/>
     </row>
     <row r="32" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="B32" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="B32" s="20" t="s">
-        <v>210</v>
-      </c>
       <c r="C32" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D32" s="20"/>
       <c r="E32" s="14"/>
@@ -5256,13 +5263,13 @@
     </row>
     <row r="33" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="B33" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="B33" s="20" t="s">
-        <v>212</v>
-      </c>
       <c r="C33" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D33" s="20"/>
       <c r="E33" s="14"/>
@@ -5319,13 +5326,13 @@
     </row>
     <row r="34" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A34" s="20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D34" s="20"/>
       <c r="E34" s="14"/>
@@ -5382,13 +5389,13 @@
     </row>
     <row r="35" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D35" s="20"/>
       <c r="E35" s="14"/>
@@ -5445,13 +5452,13 @@
     </row>
     <row r="36" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D36" s="20"/>
       <c r="E36" s="14"/>
@@ -5508,13 +5515,13 @@
     </row>
     <row r="37" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D37" s="20"/>
       <c r="E37" s="14"/>
@@ -5571,13 +5578,13 @@
     </row>
     <row r="38" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A38" s="20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D38" s="20"/>
       <c r="E38" s="14"/>
@@ -5634,13 +5641,13 @@
     </row>
     <row r="39" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A39" s="20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D39" s="20"/>
       <c r="E39" s="14"/>
@@ -5697,13 +5704,13 @@
     </row>
     <row r="40" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D40" s="20"/>
       <c r="E40" s="14"/>
@@ -5760,13 +5767,13 @@
     </row>
     <row r="41" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A41" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D41" s="20"/>
       <c r="E41" s="14"/>
@@ -5823,13 +5830,13 @@
     </row>
     <row r="42" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A42" s="20" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D42" s="20"/>
       <c r="E42" s="14"/>
@@ -5886,11 +5893,11 @@
     </row>
     <row r="43" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B43" s="14"/>
       <c r="C43" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
@@ -5947,160 +5954,160 @@
     </row>
     <row r="44" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="C44" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="E44" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="C44" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="E44" s="15" t="s">
-        <v>224</v>
-      </c>
       <c r="F44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="J44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="L44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="M44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="N44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="O44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="P44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="R44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="S44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="T44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="U44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="V44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="W44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="X44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Y44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Z44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AA44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AB44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AC44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AD44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AE44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AF44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AG44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AH44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AI44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AJ44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AK44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AL44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AM44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AN44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AO44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AP44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AQ44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AR44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AS44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AT44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AU44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AV44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AW44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AX44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AY44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AZ44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="BA44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="BB44" s="15" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -6141,118 +6148,118 @@
   <sheetData>
     <row r="1" spans="1:42" s="24" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="E1" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="F1" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="G1" s="31" t="s">
+        <v>271</v>
+      </c>
+      <c r="H1" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" s="24" t="s">
         <v>230</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="J1" s="24" t="s">
         <v>231</v>
       </c>
-      <c r="H1" s="25" t="s">
-        <v>154</v>
-      </c>
-      <c r="I1" s="24" t="s">
+      <c r="K1" s="24" t="s">
         <v>232</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="L1" s="25" t="s">
         <v>233</v>
       </c>
-      <c r="K1" s="24" t="s">
+      <c r="M1" s="25" t="s">
         <v>234</v>
       </c>
-      <c r="L1" s="25" t="s">
+      <c r="N1" s="25" t="s">
         <v>235</v>
       </c>
-      <c r="M1" s="25" t="s">
+      <c r="O1" s="25" t="s">
         <v>236</v>
       </c>
-      <c r="N1" s="25" t="s">
+      <c r="P1" s="16" t="s">
         <v>237</v>
       </c>
-      <c r="O1" s="25" t="s">
+      <c r="Q1" s="25" t="s">
         <v>238</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="R1" s="24" t="s">
         <v>239</v>
       </c>
-      <c r="Q1" s="25" t="s">
+      <c r="S1" s="24" t="s">
         <v>240</v>
       </c>
-      <c r="R1" s="24" t="s">
+      <c r="T1" s="24" t="s">
         <v>241</v>
       </c>
-      <c r="S1" s="24" t="s">
+      <c r="U1" s="24" t="s">
         <v>242</v>
       </c>
-      <c r="T1" s="24" t="s">
+      <c r="V1" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="W1" s="24" t="s">
+        <v>195</v>
+      </c>
+      <c r="X1" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="Y1" s="31" t="s">
+        <v>272</v>
+      </c>
+      <c r="Z1" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="U1" s="24" t="s">
+      <c r="AA1" s="24" t="s">
         <v>244</v>
       </c>
-      <c r="V1" s="24" t="s">
-        <v>189</v>
-      </c>
-      <c r="W1" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="X1" s="24" t="s">
-        <v>205</v>
-      </c>
-      <c r="Y1" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="Z1" s="24" t="s">
+      <c r="AB1" s="24" t="s">
         <v>245</v>
       </c>
-      <c r="AA1" s="24" t="s">
+      <c r="AC1" s="25" t="s">
         <v>246</v>
       </c>
-      <c r="AB1" s="24" t="s">
+      <c r="AD1" s="25" t="s">
+        <v>197</v>
+      </c>
+      <c r="AE1" s="24" t="s">
+        <v>202</v>
+      </c>
+      <c r="AF1" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="AG1" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="AH1" s="25" t="s">
         <v>247</v>
       </c>
-      <c r="AC1" s="25" t="s">
+      <c r="AI1" s="24" t="s">
         <v>248</v>
       </c>
-      <c r="AD1" s="25" t="s">
-        <v>198</v>
-      </c>
-      <c r="AE1" s="24" t="s">
-        <v>203</v>
-      </c>
-      <c r="AF1" s="24" t="s">
-        <v>173</v>
-      </c>
-      <c r="AG1" s="24" t="s">
-        <v>175</v>
-      </c>
-      <c r="AH1" s="25" t="s">
+      <c r="AJ1" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="AK1" s="24" t="s">
         <v>249</v>
       </c>
-      <c r="AI1" s="24" t="s">
+      <c r="AL1" s="24" t="s">
         <v>250</v>
-      </c>
-      <c r="AJ1" s="25" t="s">
-        <v>186</v>
-      </c>
-      <c r="AK1" s="24" t="s">
-        <v>251</v>
-      </c>
-      <c r="AL1" s="24" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:42" x14ac:dyDescent="0.25">
@@ -6381,17 +6388,17 @@
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="B5" s="22" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C5" s="22"/>
       <c r="F5" s="26" t="s">
+        <v>252</v>
+      </c>
+      <c r="G5" s="26" t="s">
+        <v>253</v>
+      </c>
+      <c r="H5" s="26" t="s">
         <v>254</v>
-      </c>
-      <c r="G5" s="26" t="s">
-        <v>255</v>
-      </c>
-      <c r="H5" s="26" t="s">
-        <v>256</v>
       </c>
       <c r="I5" s="26"/>
       <c r="J5" s="26"/>
@@ -6401,7 +6408,7 @@
       <c r="N5" s="26"/>
       <c r="O5" s="26"/>
       <c r="P5" s="26" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="Q5" s="26"/>
       <c r="R5" s="26"/>
@@ -6432,14 +6439,14 @@
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="B6" s="22" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C6" s="22"/>
       <c r="F6" s="26" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H6" s="26"/>
       <c r="I6" s="26"/>
@@ -6450,7 +6457,7 @@
       <c r="N6" s="26"/>
       <c r="O6" s="26"/>
       <c r="P6" s="26" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="Q6" s="26"/>
       <c r="R6" s="26"/>
@@ -6481,14 +6488,14 @@
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="B7" s="22" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C7" s="22"/>
       <c r="F7" s="26" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H7" s="26"/>
       <c r="I7" s="26"/>
@@ -6499,15 +6506,15 @@
       <c r="N7" s="26"/>
       <c r="O7" s="26"/>
       <c r="P7" s="26" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="Q7" s="26"/>
       <c r="R7" s="26"/>
       <c r="S7" s="26" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="T7" s="26" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="U7" s="26"/>
       <c r="V7" s="26"/>
@@ -6521,7 +6528,7 @@
       <c r="AD7" s="26"/>
       <c r="AE7" s="26"/>
       <c r="AF7" s="26" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="AG7" s="26"/>
       <c r="AH7" s="26"/>
@@ -6536,14 +6543,14 @@
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
       <c r="B8" s="22" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C8" s="22"/>
       <c r="F8" s="26" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H8" s="26"/>
       <c r="I8" s="26"/>
@@ -6554,7 +6561,7 @@
       <c r="N8" s="26"/>
       <c r="O8" s="26"/>
       <c r="P8" s="26" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="Q8" s="26"/>
       <c r="R8" s="26"/>
@@ -6570,15 +6577,15 @@
       <c r="AB8" s="26"/>
       <c r="AC8" s="26"/>
       <c r="AD8" s="14" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="AE8" s="26"/>
       <c r="AF8" s="26" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="AG8" s="26"/>
       <c r="AH8" s="26" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AI8" s="26"/>
       <c r="AJ8" s="26"/>

</xml_diff>

<commit_message>
use (most) question sheet column titles as in current Mapping.xlsm
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping.xlsx
+++ b/tests/testthat/excel/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D19B08-12F6-4408-80E7-9A2F0F26265B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F78E021F-AB5C-4DCF-8C0B-6927BE66933A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="275">
   <si>
     <t>Make script</t>
   </si>
@@ -521,9 +521,6 @@
     <t>q2 q3</t>
   </si>
   <si>
-    <t>Invalid</t>
-  </si>
-  <si>
     <t>Invalid values</t>
   </si>
   <si>
@@ -761,22 +758,10 @@
     <t>CatLab</t>
   </si>
   <si>
-    <t>StatRec</t>
-  </si>
-  <si>
-    <t>StatInvalid</t>
-  </si>
-  <si>
-    <t>Stat</t>
-  </si>
-  <si>
     <t>StatVar</t>
   </si>
   <si>
     <t>TitleSPSS</t>
-  </si>
-  <si>
-    <t>Footer</t>
   </si>
   <si>
     <t>Sort</t>
@@ -801,9 +786,6 @@
   </si>
   <si>
     <t>Details</t>
-  </si>
-  <si>
-    <t>MWLabel</t>
   </si>
   <si>
     <t>Mult</t>
@@ -880,6 +862,30 @@
   <si>
     <t>ColVar</t>
   </si>
+  <si>
+    <t>Unguelt</t>
+  </si>
+  <si>
+    <t>MWRec</t>
+  </si>
+  <si>
+    <t>UngueltMW</t>
+  </si>
+  <si>
+    <t>MetrMac</t>
+  </si>
+  <si>
+    <t>Fussnote</t>
+  </si>
+  <si>
+    <t>MeanOverviewLabel</t>
+  </si>
+  <si>
+    <t>RvEmp</t>
+  </si>
+  <si>
+    <t>ZsfgMW</t>
+  </si>
 </sst>
 </file>
 
@@ -888,7 +894,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yy\ hh:mm"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -938,8 +944,15 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1024,6 +1037,12 @@
         <bgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1038,7 +1057,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1083,6 +1102,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2523,7 +2543,7 @@
     </row>
     <row r="5" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A5" s="28" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>150</v>
@@ -2590,16 +2610,16 @@
     </row>
     <row r="6" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A6" s="28" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B6" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="D6" s="20" t="s">
         <v>155</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>156</v>
       </c>
       <c r="E6" s="14">
         <v>-1</v>
@@ -2755,13 +2775,13 @@
     </row>
     <row r="7" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="C7" s="20" t="s">
         <v>158</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>159</v>
       </c>
       <c r="D7" s="20"/>
       <c r="E7" s="14">
@@ -2918,13 +2938,13 @@
     </row>
     <row r="8" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>161</v>
-      </c>
       <c r="C8" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D8" s="20"/>
       <c r="E8" s="14">
@@ -3081,19 +3101,19 @@
     </row>
     <row r="9" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B9" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="D9" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="D9" s="20" t="s">
-        <v>164</v>
-      </c>
       <c r="E9" s="14" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
@@ -3205,14 +3225,14 @@
     </row>
     <row r="11" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" s="20" t="s">
         <v>165</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>166</v>
       </c>
       <c r="C11" s="20"/>
       <c r="D11" s="20" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
@@ -3268,11 +3288,11 @@
     </row>
     <row r="12" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D12" s="20"/>
       <c r="E12" s="14"/>
@@ -3329,10 +3349,10 @@
     </row>
     <row r="13" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>169</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>170</v>
       </c>
       <c r="C13" s="20"/>
       <c r="D13" s="20"/>
@@ -3390,11 +3410,11 @@
     </row>
     <row r="14" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D14" s="20"/>
       <c r="E14" s="14"/>
@@ -3451,10 +3471,10 @@
     </row>
     <row r="15" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>172</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>173</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
@@ -3512,14 +3532,14 @@
     </row>
     <row r="16" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A16" s="20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B16" s="20"/>
       <c r="C16" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E16" s="14"/>
       <c r="F16" s="14"/>
@@ -3575,10 +3595,10 @@
     </row>
     <row r="17" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17" s="20" t="s">
         <v>176</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>177</v>
       </c>
       <c r="C17" s="20"/>
       <c r="D17" s="20"/>
@@ -3636,335 +3656,335 @@
     </row>
     <row r="18" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="B18" s="20" t="s">
         <v>178</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="C18" s="20" t="s">
         <v>179</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>180</v>
       </c>
       <c r="D18" s="20"/>
       <c r="E18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="M18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Q18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="R18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="S18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="T18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="U18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="V18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="W18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="X18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Y18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="Z18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AA18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AB18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AC18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AD18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AE18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AF18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AG18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AH18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AI18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AJ18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AK18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AL18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AM18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AN18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AO18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AP18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AQ18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AR18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AS18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AT18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AU18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AV18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AW18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AX18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AY18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AZ18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BA18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BB18" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BD18" s="19"/>
     </row>
     <row r="19" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D19" s="20"/>
       <c r="E19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="L19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="M19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="N19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="P19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Q19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="R19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="S19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="T19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="U19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="W19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="X19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Y19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="Z19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AA19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AB19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AC19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AD19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AE19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AF19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AG19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AH19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AI19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AJ19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AK19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AL19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AM19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AN19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AO19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AP19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AQ19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AR19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AS19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AT19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AU19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AV19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AW19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AX19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AY19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AZ19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="BA19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="BB19" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="BD19" s="19"/>
     </row>
     <row r="20" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D20" s="20"/>
       <c r="E20" s="14"/>
@@ -4021,175 +4041,175 @@
     </row>
     <row r="21" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B21" s="20" t="s">
         <v>185</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>186</v>
       </c>
       <c r="C21" s="20"/>
       <c r="D21" s="20"/>
       <c r="E21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="L21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Q21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="R21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="S21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="T21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="U21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="V21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="W21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="X21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Y21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Z21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AA21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AB21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AC21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AD21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AE21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AF21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AG21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AH21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AI21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AJ21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AK21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AL21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AM21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AN21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AO21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AP21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AQ21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AR21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AS21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AT21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AU21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AV21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AW21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AX21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AY21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AZ21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="BA21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="BB21" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="BD21" s="19"/>
     </row>
     <row r="22" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="B22" s="20" t="s">
         <v>188</v>
-      </c>
-      <c r="B22" s="20" t="s">
-        <v>189</v>
       </c>
       <c r="C22" s="20"/>
       <c r="D22" s="20" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E22" s="14"/>
       <c r="F22" s="14"/>
@@ -4245,11 +4265,11 @@
     </row>
     <row r="23" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B23" s="20"/>
       <c r="C23" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D23" s="20"/>
       <c r="E23" s="14"/>
@@ -4306,11 +4326,11 @@
     </row>
     <row r="24" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B24" s="20"/>
       <c r="C24" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D24" s="20"/>
       <c r="E24" s="14"/>
@@ -4367,11 +4387,11 @@
     </row>
     <row r="25" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B25" s="20"/>
       <c r="C25" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D25" s="20"/>
       <c r="E25" s="14"/>
@@ -4428,11 +4448,11 @@
     </row>
     <row r="26" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B26" s="20"/>
       <c r="C26" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D26" s="20"/>
       <c r="E26" s="14"/>
@@ -4489,498 +4509,498 @@
     </row>
     <row r="27" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D27" s="20"/>
       <c r="E27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="M27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="N27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="O27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="Q27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="R27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="S27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="T27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="U27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="V27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="W27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="X27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="Y27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="Z27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AA27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AB27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AC27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AD27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AE27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AF27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AG27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AH27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AI27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AJ27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AK27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AL27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AM27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AN27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AO27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AP27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AQ27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AR27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AS27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AT27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AU27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AV27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AW27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AX27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AY27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="AZ27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="BA27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="BB27" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="BD27" s="19"/>
     </row>
     <row r="28" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
+        <v>196</v>
+      </c>
+      <c r="B28" s="20" t="s">
         <v>197</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="C28" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="D28" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="E28" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="E28" s="14" t="s">
-        <v>201</v>
-      </c>
       <c r="F28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="M28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="N28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="P28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Q28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="R28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="S28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="T28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="U28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="V28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="W28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="X28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Y28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Z28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AA28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AB28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AC28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AD28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AE28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AF28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AG28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AH28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AI28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AJ28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AK28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AL28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AM28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AN28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AO28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AP28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AQ28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AR28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AS28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AT28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AU28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AV28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AW28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AX28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AY28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AZ28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="BA28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="BB28" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="BD28" s="19"/>
     </row>
     <row r="29" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B29" s="20"/>
       <c r="C29" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D29" s="20"/>
       <c r="E29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="K29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="N29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="O29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="P29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Q29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="R29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="S29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="T29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="U29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="V29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="W29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="X29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Y29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Z29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AA29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AB29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AC29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AD29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AE29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AF29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AG29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AH29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AI29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AJ29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AK29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AL29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AM29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AN29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AO29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AP29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AQ29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AR29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AS29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AT29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AU29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AV29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AW29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AX29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AY29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AZ29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="BA29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="BB29" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="BD29" s="19"/>
     </row>
     <row r="30" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D30" s="20"/>
       <c r="E30" s="14"/>
@@ -5037,176 +5057,176 @@
     </row>
     <row r="31" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="B31" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="B31" s="20" t="s">
-        <v>206</v>
-      </c>
       <c r="C31" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D31" s="20"/>
       <c r="E31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="L31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="M31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="O31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="P31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="Q31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="R31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="S31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="T31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="U31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="V31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="W31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="X31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="Y31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="Z31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AA31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AB31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AC31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AD31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AE31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AF31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AG31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AH31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AI31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AJ31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AK31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AL31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AM31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AN31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AO31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AP31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AQ31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AR31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AS31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AT31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AU31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AV31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AW31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AX31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AY31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AZ31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="BA31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="BB31" s="14" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="BD31" s="19"/>
     </row>
     <row r="32" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="B32" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="B32" s="20" t="s">
-        <v>209</v>
-      </c>
       <c r="C32" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D32" s="20"/>
       <c r="E32" s="14"/>
@@ -5263,13 +5283,13 @@
     </row>
     <row r="33" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="B33" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="B33" s="20" t="s">
-        <v>211</v>
-      </c>
       <c r="C33" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D33" s="20"/>
       <c r="E33" s="14"/>
@@ -5326,13 +5346,13 @@
     </row>
     <row r="34" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A34" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D34" s="20"/>
       <c r="E34" s="14"/>
@@ -5389,13 +5409,13 @@
     </row>
     <row r="35" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D35" s="20"/>
       <c r="E35" s="14"/>
@@ -5452,13 +5472,13 @@
     </row>
     <row r="36" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D36" s="20"/>
       <c r="E36" s="14"/>
@@ -5515,13 +5535,13 @@
     </row>
     <row r="37" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D37" s="20"/>
       <c r="E37" s="14"/>
@@ -5578,13 +5598,13 @@
     </row>
     <row r="38" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A38" s="20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D38" s="20"/>
       <c r="E38" s="14"/>
@@ -5641,13 +5661,13 @@
     </row>
     <row r="39" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A39" s="20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D39" s="20"/>
       <c r="E39" s="14"/>
@@ -5704,13 +5724,13 @@
     </row>
     <row r="40" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D40" s="20"/>
       <c r="E40" s="14"/>
@@ -5767,13 +5787,13 @@
     </row>
     <row r="41" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A41" s="20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D41" s="20"/>
       <c r="E41" s="14"/>
@@ -5830,13 +5850,13 @@
     </row>
     <row r="42" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A42" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D42" s="20"/>
       <c r="E42" s="14"/>
@@ -5893,11 +5913,11 @@
     </row>
     <row r="43" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B43" s="14"/>
       <c r="C43" s="20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
@@ -5954,160 +5974,160 @@
     </row>
     <row r="44" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="C44" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E44" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="C44" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="E44" s="15" t="s">
-        <v>223</v>
-      </c>
       <c r="F44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="I44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="K44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="L44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="M44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="O44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="P44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Q44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="R44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="S44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="T44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="U44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="V44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="W44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="X44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Y44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Z44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AA44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AB44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AC44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AD44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AE44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AF44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AG44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AH44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AI44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AJ44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AK44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AL44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AM44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AN44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AO44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AP44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AQ44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AR44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AS44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AT44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AU44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AV44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AW44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AX44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AY44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AZ44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BA44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="BB44" s="15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -6148,118 +6168,118 @@
   <sheetData>
     <row r="1" spans="1:42" s="24" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>225</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="E1" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="F1" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="G1" s="31" t="s">
+        <v>265</v>
+      </c>
+      <c r="H1" s="25" t="s">
+        <v>267</v>
+      </c>
+      <c r="I1" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="J1" s="24" t="s">
+        <v>230</v>
+      </c>
+      <c r="K1" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="L1" s="25" t="s">
+        <v>268</v>
+      </c>
+      <c r="M1" s="25" t="s">
+        <v>269</v>
+      </c>
+      <c r="N1" s="25" t="s">
+        <v>270</v>
+      </c>
+      <c r="O1" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="P1" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q1" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="H1" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="I1" s="24" t="s">
-        <v>230</v>
-      </c>
-      <c r="J1" s="24" t="s">
-        <v>231</v>
-      </c>
-      <c r="K1" s="24" t="s">
-        <v>232</v>
-      </c>
-      <c r="L1" s="25" t="s">
-        <v>233</v>
-      </c>
-      <c r="M1" s="25" t="s">
+      <c r="R1" s="24" t="s">
         <v>234</v>
       </c>
-      <c r="N1" s="25" t="s">
+      <c r="S1" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="O1" s="25" t="s">
+      <c r="T1" s="24" t="s">
         <v>236</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="U1" s="24" t="s">
         <v>237</v>
       </c>
-      <c r="Q1" s="25" t="s">
+      <c r="V1" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="W1" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="X1" s="24" t="s">
+        <v>203</v>
+      </c>
+      <c r="Y1" s="31" t="s">
+        <v>266</v>
+      </c>
+      <c r="Z1" s="24" t="s">
         <v>238</v>
       </c>
-      <c r="R1" s="24" t="s">
+      <c r="AA1" s="24" t="s">
         <v>239</v>
       </c>
-      <c r="S1" s="24" t="s">
+      <c r="AB1" s="24" t="s">
         <v>240</v>
       </c>
-      <c r="T1" s="24" t="s">
+      <c r="AC1" s="25" t="s">
         <v>241</v>
       </c>
-      <c r="U1" s="24" t="s">
+      <c r="AD1" s="25" t="s">
+        <v>274</v>
+      </c>
+      <c r="AE1" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="AF1" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="AG1" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="AH1" s="32" t="s">
+        <v>272</v>
+      </c>
+      <c r="AI1" s="24" t="s">
         <v>242</v>
       </c>
-      <c r="V1" s="24" t="s">
-        <v>188</v>
-      </c>
-      <c r="W1" s="24" t="s">
-        <v>195</v>
-      </c>
-      <c r="X1" s="24" t="s">
-        <v>204</v>
-      </c>
-      <c r="Y1" s="31" t="s">
-        <v>272</v>
-      </c>
-      <c r="Z1" s="24" t="s">
+      <c r="AJ1" s="32" t="s">
+        <v>273</v>
+      </c>
+      <c r="AK1" s="24" t="s">
         <v>243</v>
       </c>
-      <c r="AA1" s="24" t="s">
+      <c r="AL1" s="24" t="s">
         <v>244</v>
-      </c>
-      <c r="AB1" s="24" t="s">
-        <v>245</v>
-      </c>
-      <c r="AC1" s="25" t="s">
-        <v>246</v>
-      </c>
-      <c r="AD1" s="25" t="s">
-        <v>197</v>
-      </c>
-      <c r="AE1" s="24" t="s">
-        <v>202</v>
-      </c>
-      <c r="AF1" s="24" t="s">
-        <v>172</v>
-      </c>
-      <c r="AG1" s="24" t="s">
-        <v>174</v>
-      </c>
-      <c r="AH1" s="25" t="s">
-        <v>247</v>
-      </c>
-      <c r="AI1" s="24" t="s">
-        <v>248</v>
-      </c>
-      <c r="AJ1" s="25" t="s">
-        <v>185</v>
-      </c>
-      <c r="AK1" s="24" t="s">
-        <v>249</v>
-      </c>
-      <c r="AL1" s="24" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:42" x14ac:dyDescent="0.25">
@@ -6388,17 +6408,17 @@
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="B5" s="22" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C5" s="22"/>
       <c r="F5" s="26" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="I5" s="26"/>
       <c r="J5" s="26"/>
@@ -6408,7 +6428,7 @@
       <c r="N5" s="26"/>
       <c r="O5" s="26"/>
       <c r="P5" s="26" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="Q5" s="26"/>
       <c r="R5" s="26"/>
@@ -6439,14 +6459,14 @@
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="B6" s="22" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C6" s="22"/>
       <c r="F6" s="26" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H6" s="26"/>
       <c r="I6" s="26"/>
@@ -6457,7 +6477,7 @@
       <c r="N6" s="26"/>
       <c r="O6" s="26"/>
       <c r="P6" s="26" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="Q6" s="26"/>
       <c r="R6" s="26"/>
@@ -6488,14 +6508,14 @@
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="B7" s="22" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C7" s="22"/>
       <c r="F7" s="26" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H7" s="26"/>
       <c r="I7" s="26"/>
@@ -6506,15 +6526,15 @@
       <c r="N7" s="26"/>
       <c r="O7" s="26"/>
       <c r="P7" s="26" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="Q7" s="26"/>
       <c r="R7" s="26"/>
       <c r="S7" s="26" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="T7" s="26" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="U7" s="26"/>
       <c r="V7" s="26"/>
@@ -6528,7 +6548,7 @@
       <c r="AD7" s="26"/>
       <c r="AE7" s="26"/>
       <c r="AF7" s="26" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="AG7" s="26"/>
       <c r="AH7" s="26"/>
@@ -6543,14 +6563,14 @@
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
       <c r="B8" s="22" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="C8" s="22"/>
       <c r="F8" s="26" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="H8" s="26"/>
       <c r="I8" s="26"/>
@@ -6561,7 +6581,7 @@
       <c r="N8" s="26"/>
       <c r="O8" s="26"/>
       <c r="P8" s="26" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="Q8" s="26"/>
       <c r="R8" s="26"/>
@@ -6577,15 +6597,15 @@
       <c r="AB8" s="26"/>
       <c r="AC8" s="26"/>
       <c r="AD8" s="14" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="AE8" s="26"/>
       <c r="AF8" s="26" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="AG8" s="26"/>
       <c r="AH8" s="26" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="AI8" s="26"/>
       <c r="AJ8" s="26"/>

</xml_diff>

<commit_message>
also put new named region V_XMLName in this mapping
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping.xlsx
+++ b/tests/testthat/excel/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5D921BD-5AAF-4513-9F2E-3DB5C4DEE3E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2273012-6F2E-4BB5-A78F-8672CA49D57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -32,14 +32,15 @@
     <definedName name="V_Language">Config!$B$15</definedName>
     <definedName name="V_Lexikon">[2]Lexikon!$A$2:$H$192</definedName>
     <definedName name="V_Namenszusatz">Config!$B$17</definedName>
-    <definedName name="V_Projektleiter">Config!$B$38</definedName>
-    <definedName name="V_ProjektleiterCol">Config!$C$38</definedName>
+    <definedName name="V_Projektleiter">Config!$B$39</definedName>
+    <definedName name="V_ProjektleiterCol">Config!$C$39</definedName>
     <definedName name="V_Projektname">Config!$B$21</definedName>
     <definedName name="V_Projektverzeichnis">Config!$B$20</definedName>
     <definedName name="V_Scenario">Config!$B$16</definedName>
     <definedName name="V_ScenDetail">[1]Macro!$E$3:$BB$43</definedName>
     <definedName name="V_ScenName">Config!$C$16</definedName>
-    <definedName name="V_TemplatePath">Config!$B$26</definedName>
+    <definedName name="V_TemplatePath">Config!$B$27</definedName>
+    <definedName name="V_XMLName">Config!$B$23</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,6 +63,29 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Wolf Wilke</author>
+  </authors>
+  <commentList>
+    <comment ref="A23" authorId="0" shapeId="0" xr:uid="{E5B4CAE9-8D0E-4066-ACEF-1DBC18426B4B}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Name of XML file with table date, to be appended by '&lt;QuestNo&gt;.xml'</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>wolf</author>
@@ -162,7 +186,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="279">
   <si>
     <t>Make script</t>
   </si>
@@ -994,6 +1018,12 @@
   <si>
     <t>Exclusive</t>
   </si>
+  <si>
+    <t>XML name</t>
+  </si>
+  <si>
+    <t>dev\xml\XML_test_Draft_</t>
+  </si>
 </sst>
 </file>
 
@@ -1002,7 +1032,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yy\ hh:mm"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1072,8 +1102,13 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1152,6 +1187,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1166,7 +1207,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1204,29 +1245,20 @@
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1459,7 +1491,7 @@
         <xdr:cNvPr id="2" name="TabellenErzeugen">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2C11E0F-9396-4723-9E7C-DCA9D4511292}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1504,7 +1536,7 @@
         <xdr:cNvPr id="3" name="AusgewaehlteTabellenErzeugen">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A72DB92-A95C-4C5A-B740-37C67FD3C8F4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1538,14 +1570,19 @@
   </xdr:oneCellAnchor>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
+      <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>6</xdr:col>
           <xdr:colOff>800100</xdr:colOff>
           <xdr:row>0</xdr:row>
           <xdr:rowOff>47625</xdr:rowOff>
         </xdr:from>
-        <xdr:ext cx="1524000" cy="180975"/>
+        <xdr:to>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>2324100</xdr:colOff>
+          <xdr:row>0</xdr:row>
+          <xdr:rowOff>228600</xdr:rowOff>
+        </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2049" name="Drop Down 1" hidden="1">
@@ -1554,7 +1591,7 @@
                   <a14:compatExt spid="_x0000_s2049"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F035105D-BD67-4ACB-BB4D-6FBDB13AB3DA}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000001080000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1585,7 +1622,7 @@
           </xdr:spPr>
         </xdr:sp>
         <xdr:clientData/>
-      </xdr:oneCellAnchor>
+      </xdr:twoCellAnchor>
     </mc:Choice>
     <mc:Fallback/>
   </mc:AlternateContent>
@@ -2038,8 +2075,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ44"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AMJ45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" style="1" customWidth="1"/>
@@ -2260,18 +2297,16 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="10" t="e">
-        <f>#N/A</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F23" s="13"/>
+      <c r="A23" s="32" t="s">
+        <v>277</v>
+      </c>
+      <c r="B23" s="32" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B24" s="10" t="e">
         <f>#N/A</f>
@@ -2280,138 +2315,149 @@
       <c r="F24" s="13"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="10" t="e">
+        <f>#N/A</f>
+        <v>#N/A</v>
+      </c>
       <c r="F25" s="13"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+      <c r="F26" s="13"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B27" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="F26" s="13"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
+      <c r="F27" s="13"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>31</v>
-      </c>
+      <c r="A28" s="10"/>
+      <c r="B28" s="10"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B31" s="10" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B32" s="7" t="b">
-        <f>FALSE()</f>
-        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="B33" s="7" t="b">
         <f>FALSE()</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B35" s="14">
-        <v>100</v>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="7" t="b">
+        <f>FALSE()</f>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="14" t="s">
+      <c r="B37" s="14" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C37" s="10" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C38" s="10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B39" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C38" s="1">
+      <c r="C39" s="1">
         <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="10" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="10" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>H5&lt;H3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>H7&lt;H5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>H9&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2594,8 +2640,8 @@
     </row>
     <row r="2" spans="1:56" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:56" s="18" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30"/>
+      <c r="A3" s="30"/>
+      <c r="B3" s="31"/>
       <c r="E3" s="18">
         <v>1</v>
       </c>
@@ -2749,8 +2795,8 @@
       <c r="BD3" s="19"/>
     </row>
     <row r="4" spans="1:56" s="18" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="29"/>
-      <c r="B4" s="30"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="31"/>
       <c r="E4" s="18" t="s">
         <v>16</v>
       </c>
@@ -6547,7 +6593,7 @@
       <c r="F1" s="28" t="s">
         <v>225</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="29" t="s">
         <v>257</v>
       </c>
       <c r="H1" s="28" t="s">
@@ -33785,11 +33831,11 @@
       <c r="AP678" s="26"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
only put q2 ColVar in mapping file
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping.xlsx
+++ b/tests/testthat/excel/mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2273012-6F2E-4BB5-A78F-8672CA49D57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869BAFE7-0783-4528-B38C-18F0AFE4BCD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -1246,13 +1246,13 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1714,6 +1714,7 @@
       <sheetName val="TableDefinition"/>
       <sheetName val="Free Beispiele"/>
       <sheetName val="Limesurvey"/>
+      <sheetName val="Funktionen 202304"/>
     </sheetNames>
     <definedNames>
       <definedName name="SF40_KlickenSieAuf"/>
@@ -1732,6 +1733,7 @@
       <sheetData sheetId="7"/>
       <sheetData sheetId="8"/>
       <sheetData sheetId="9"/>
+      <sheetData sheetId="10" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1746,16 +1748,17 @@
     <sheetNames>
       <sheetName val="Config"/>
       <sheetName val="Data"/>
+      <sheetName val="Free0"/>
       <sheetName val="Variables"/>
+      <sheetName val="Verbatims"/>
       <sheetName val="Label"/>
-      <sheetName val="Verbatims"/>
-      <sheetName val="VerbCode"/>
       <sheetName val="Free1"/>
       <sheetName val="Free2"/>
       <sheetName val="Macro"/>
       <sheetName val="Questions"/>
       <sheetName val="Log10"/>
       <sheetName val="Log20"/>
+      <sheetName val="Diff"/>
       <sheetName val="Log40"/>
       <sheetName val="Tabelle1"/>
     </sheetNames>
@@ -1774,6 +1777,7 @@
       <sheetData sheetId="11"/>
       <sheetData sheetId="12"/>
       <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2297,10 +2301,10 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="30" t="s">
         <v>277</v>
       </c>
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="30" t="s">
         <v>278</v>
       </c>
     </row>
@@ -2640,8 +2644,8 @@
     </row>
     <row r="2" spans="1:56" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:56" s="18" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="30"/>
-      <c r="B3" s="31"/>
+      <c r="A3" s="31"/>
+      <c r="B3" s="32"/>
       <c r="E3" s="18">
         <v>1</v>
       </c>
@@ -2795,8 +2799,8 @@
       <c r="BD3" s="19"/>
     </row>
     <row r="4" spans="1:56" s="18" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="30"/>
-      <c r="B4" s="31"/>
+      <c r="A4" s="31"/>
+      <c r="B4" s="32"/>
       <c r="E4" s="18" t="s">
         <v>16</v>
       </c>
@@ -2963,7 +2967,7 @@
         <v>152</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>152</v>
+        <v>240</v>
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>

</xml_diff>